<commit_message>
feat: append tasa_aplicada column to cash flow output
* Add `tasa_aplicada` tracking in `calculate_interest_flow`
* Retain `tasa_aplicada` when merging independent amortization schedules with NA padding
* Export `tasa_aplicada` explicitly to final xlsx flow

Co-authored-by: pguzman201510-maker <226378331+pguzman201510-maker@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test_out.xlsx
+++ b/test_out.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,6 +451,11 @@
           <t>pago_interes</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>tasa_aplicada</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -477,6 +482,7 @@
       <c r="F2" t="n">
         <v>5</v>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -503,6 +509,7 @@
       <c r="F3" t="n">
         <v>4</v>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: append CLASE_INT and tipo_tasa categorization to cash flow
* Append `CLASE_INT` explicitly to the consolidated output tracking the exact rate class
* Generate and append `tipo_tasa` boolean column identifying if the credit employs a FIJA or VARIABLE structure based on the central config rules
* Update `exporter.py` to persist these new identifier columns through the final output `.xlsx` file

Co-authored-by: pguzman201510-maker <226378331+pguzman201510-maker@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test_out.xlsx
+++ b/test_out.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,20 +438,30 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>CLASE_INT</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>tipo_tasa</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>fecha_operacion</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>pago_amortizacion</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>pago_interes</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tasa_aplicada</t>
         </is>
@@ -473,16 +483,18 @@
           <t>BID</t>
         </is>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>100</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>5</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -500,16 +512,18 @@
           <t>BID</t>
         </is>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>100</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>4</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>